<commit_message>
Products Search amd details
</commit_message>
<xml_diff>
--- a/testdata/TutorialninjaLoginData.xlsx
+++ b/testdata/TutorialninjaLoginData.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\EclipseProjects\Tutorialninja\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E0CDE7-6EB3-4B5A-ACB6-F96226B055DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292F32D8-9CB7-4E92-8FF2-FF856C91793B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="Search" sheetId="2" r:id="rId2"/>
+    <sheet name="Products" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>Username</t>
   </si>
@@ -55,6 +57,39 @@
   </si>
   <si>
     <t>Invalid</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>SubCategory</t>
+  </si>
+  <si>
+    <t>Desktops</t>
+  </si>
+  <si>
+    <t>Mac (1)</t>
+  </si>
+  <si>
+    <t>Tablets</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>Search</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>Mac</t>
+  </si>
+  <si>
+    <t>caa</t>
+  </si>
+  <si>
+    <t>ca</t>
   </si>
 </sst>
 </file>
@@ -600,4 +635,84 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EDA792C-20EB-45E9-B46B-F9D578FACE51}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF1F27C-DFBD-4A9C-AB05-78D0A6604ECD}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.109375" customWidth="1"/>
+    <col min="2" max="2" width="28.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>